<commit_message>
docs: note both AR/FR receipt templates now exist
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/livraisonAR.xlsx
+++ b/frontend/public/templates/livraisonAR.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>الســــــــــــلعة الـــمفصلة الآتيـــــــــــة</t>
   </si>
@@ -67,24 +67,19 @@
   </si>
   <si>
     <t>totalttc</t>
+  </si>
+  <si>
+    <t>وصل تسليم</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -190,7 +185,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -208,8 +203,14 @@
         <fgColor indexed="30"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="34">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -662,144 +663,158 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="13" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -816,82 +831,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>323851</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Round Same Side Corner Rectangle 6"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3486150" y="9525"/>
-          <a:ext cx="1009650" cy="314326"/>
-        </a:xfrm>
-        <a:prstGeom prst="round2SameRect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr" anchorCtr="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="ar-DZ" sz="1600" b="1">
-              <a:latin typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-              <a:cs typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-            </a:rPr>
-            <a:t>وصل</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ar-DZ" sz="1600" b="1" baseline="0">
-              <a:latin typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-              <a:cs typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-            </a:rPr>
-            <a:t> تسليم</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1600" b="1">
-            <a:latin typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-            <a:cs typeface="ae_AlMateen" panose="02060803050605020204" pitchFamily="18" charset="-78"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1173,251 +1112,274 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="17" t="s">
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="1"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="40"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="18" t="s">
+      <c r="A3" s="36"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="43"/>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
+      <c r="A5" s="39"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="43"/>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
+      <c r="A6" s="39"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="45"/>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="46"/>
-      <c r="I7" s="46"/>
-      <c r="J7" s="47"/>
+      <c r="A7" s="41"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="43"/>
     </row>
     <row r="8" spans="1:11" ht="22.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="37" t="s">
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="6"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="5"/>
     </row>
     <row r="9" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
     </row>
     <row r="10" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="24" t="s">
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="H10" s="25"/>
-      <c r="I10" s="20" t="s">
+      <c r="H10" s="21"/>
+      <c r="I10" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="J10" s="21"/>
-      <c r="K10" s="7"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="7"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="12"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="44"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="12"/>
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="44"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="44"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="12"/>
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="44"/>
     </row>
     <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="12"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="44"/>
     </row>
     <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="12"/>
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="44"/>
     </row>
     <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12" t="s">
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="H17" s="12"/>
-      <c r="I17" s="13" t="s">
+      <c r="H17" s="44"/>
+      <c r="I17" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="J17" s="12"/>
+      <c r="J17" s="44"/>
     </row>
     <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12" t="s">
+      <c r="A18" s="44"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="H18" s="12"/>
-      <c r="I18" s="13" t="s">
+      <c r="H18" s="44"/>
+      <c r="I18" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="J18" s="12"/>
+      <c r="J18" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="35">
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="A17:F18"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:J13"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="E1:G1"/>
     <mergeCell ref="E3:J6"/>
@@ -1432,29 +1394,9 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:D6"/>
     <mergeCell ref="A7:J7"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="A17:F18"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="H1:J1"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="11" scale="87" fitToHeight="0" orientation="portrait" copies="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="11" scale="87" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>